<commit_message>
optimised twitter engagement legacy sql query
</commit_message>
<xml_diff>
--- a/test/test_logbook.xlsx
+++ b/test/test_logbook.xlsx
@@ -1464,7 +1464,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2025-11-09 21:36:03</t>
+          <t>2025-11-11 17:49:55</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2025-11-09 21:36:03</t>
+          <t>2025-11-11 17:49:55</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2025-11-09 21:35:42</t>
+          <t>2025-11-11 17:21:17</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2025-11-09 21:35:55</t>
+          <t>2025-11-11 17:49:40</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2025-11-09 21:35:55</t>
+          <t>2025-11-11 17:49:40</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2025-11-09 21:35:56</t>
+          <t>2025-11-11 17:49:41</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2025-11-09 21:35:56</t>
+          <t>2025-11-11 17:49:41</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2025-11-09 21:35:56</t>
+          <t>2025-11-11 17:49:41</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">

</xml_diff>

<commit_message>
adding testing of logfiles and instagram outlier testing
</commit_message>
<xml_diff>
--- a/test/test_logbook.xlsx
+++ b/test/test_logbook.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -884,7 +884,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2025-11-21 16:05:52</t>
+          <t>2025-11-23 10:10:29</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-21/1_INS_engagements_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/1_INS_engagements_issue_list.csv</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2025-11-21 16:05:52</t>
+          <t>2025-11-23 10:10:30</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-21/2_INS_engagements_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/2_INS_engagements_issue_list.csv</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -948,17 +948,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2025-11-21 16:05:52</t>
+          <t>2025-11-23 10:10:30</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>fail</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>no file created :)</t>
+          <t>../test/issue_lists_2025-11-23/3_INS_engagements_issue_list.csv</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Check no missing values in weekly_reach column from redshift returned</t>
+          <t>Check no missing values in metric columns from redshift returned</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2025-11-21 16:05:52</t>
+          <t>2025-11-23 10:10:30</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2025-11-21 16:23:13</t>
+          <t>2025-11-23 10:12:29</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1044,27 +1044,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2025-11-21 16:23:13</t>
+          <t>2025-11-23 12:27:39</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>fail</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>no file created :)</t>
+          <t>../test/issue_lists_2025-11-23/6_INS_engagements_issue_list.csv</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>testing inner join - dataloss between two tables</t>
+          <t>testing missing elements in columns</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>adding views to reels plays</t>
+          <t>Check that all page IDs are found in SQL</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2025-11-21 18:15:58</t>
+          <t>2025-11-23 10:09:25</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-21/1_INS_country_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/1_INS_country_issue_list.csv</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2025-11-21 18:15:58</t>
+          <t>2025-11-23 10:09:26</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-21/2_INS_country_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/2_INS_country_issue_list.csv</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2025-11-21 18:15:59</t>
+          <t>2025-11-23 10:09:26</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2025-11-21 18:15:59</t>
+          <t>2025-11-23 10:09:26</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-21/4_INS_country_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/4_INS_country_issue_list.csv</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2025-11-21 18:15:59</t>
+          <t>2025-11-23 10:09:26</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-21/5_INS_country_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/5_INS_country_issue_list.csv</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2025-11-21 18:15:59</t>
+          <t>2025-11-23 10:09:27</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2025-11-21 18:16:02</t>
+          <t>2025-11-23 10:09:29</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2025-11-22 13:22:06</t>
+          <t>2025-11-23 10:50:17</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2025-11-22 13:22:08</t>
+          <t>2025-11-23 10:50:19</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-22/3_TWI_combination_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/3_TWI_combination_issue_list.csv</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2025-11-22 13:22:07</t>
+          <t>2025-11-23 10:50:18</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-22/2_TWI_combination_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/2_TWI_combination_issue_list.csv</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2025-11-22 13:58:47</t>
+          <t>2025-11-23 10:50:36</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-22/1_YT-_country_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/1_YT-_country_issue_list.csv</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2025-11-22 13:58:48</t>
+          <t>2025-11-23 10:50:37</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-22/2_YT-_country_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/2_YT-_country_issue_list.csv</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2025-11-22 13:58:48</t>
+          <t>2025-11-23 10:50:37</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>../test/issue_lists_2025-11-22/3_YT-_country_issue_list.csv</t>
+          <t>../test/issue_lists_2025-11-23/3_YT-_country_issue_list.csv</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2025-11-22 13:58:49</t>
+          <t>2025-11-23 10:50:37</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2025-11-22 13:58:49</t>
+          <t>2025-11-23 10:50:38</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2025-11-22 13:58:49</t>
+          <t>2025-11-23 10:50:38</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2041,6 +2041,1798 @@
       <c r="F51" t="inlineStr">
         <is>
           <t>calculating % country</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>0</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:36</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Testing if lookup DataFrame is empty</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring week tester is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>1</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:36</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring week tester is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:37</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Testing missing values in lookup</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring week tester is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>3</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:37</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Testing if lookup DataFrame is empty</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring social media accounts is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>4</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:37</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/4_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring social media accounts is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>5</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:37</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/5_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Testing missing values in lookup</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring social media accounts is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>6</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2025-11-23 11:36:47</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Testing if lookup DataFrame is empty</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring social media accounts is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>7</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2025-11-23 11:36:47</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring social media accounts is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>8</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2025-11-23 11:36:48</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Testing missing values in lookup</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring social media accounts is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>6_FBE_engagements</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:05:39</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/6_FBE_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>testing missing elements in columns</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Check that all page IDs are found in SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>7_FBE_engagements</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:05:40</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/7_FBE_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Weeks presence per account</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Check all weeks present for each account</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>8_FBE_engagements</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:05:40</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/8_FBE_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Check for NaN and positive values</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Check no missing values in engaged_reach column from redshift returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>9_FBE_engagements</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:05:40</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Check no duplicates from redshift returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>10_FBE_engagements</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:05:40</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>testing inner join - dataloss between two tables</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>checking social media accounts in lookup, adding service</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>9_FBE_country</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:07:50</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/9_FBE_country_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>testing missing elements in columns</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Check that all page IDs are found in SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>10_FBE_country</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:07:51</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/10_FBE_country_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Weeks presence per account</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Check all weeks present for each account</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>11_FBE_country</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:07:51</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Check for NaN and positive values</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Check no missing values in page fans column from redshift returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>12_FBE_country</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:07:51</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/12_FBE_country_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Check no duplicates from redshift returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>13_FBE_country</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:07:52</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/13_FBE_country_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>testing inner join - dataloss between two tables</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>calculating country %</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>14_FBE_country</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:07:52</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>testing inner join - dataloss between two tables</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>calculating country %</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>15_FBE_country</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:07:52</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>testing country percentage</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>summing country % per week &amp; account</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>7_INS_engagements</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:40</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/7_INS_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Weeks presence per account</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Check all weeks present for each account</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>6_TWI_engagements</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:25:33</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/6_TWI_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>testing missing elements in columns</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Check that all page IDs are found in SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>7_TWI_engagements</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:25:33</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/7_TWI_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Weeks presence per account</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Check all weeks present for each account</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>8_TWI_engagements</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:25:33</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/8_TWI_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Check for NaN and positive values</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Check no missing values in metric columns column from redshift returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>9_TWI_engagements</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:25:33</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Check no duplicates from redshift returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1_YT_1</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:37:27</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/1_YT_1_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>all weeks in dataset</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>testing automated extracts</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1_YT_2</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:40:12</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/1_YT_2_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>testing missing elements in columns</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>combine CMS &amp; non CMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1_YT_3</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:40:12</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/1_YT_3_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Weeks presence per account</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>combine CMS &amp; non CMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1_YT_4</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:40:12</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>combine CMS &amp; non CMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1_YT_5</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:40:12</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>testing merge row count</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>combine CMS &amp; non CMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>7_YT-_engagements</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:44:08</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/7_YT-_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>testing missing elements in columns</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>combine CMS &amp; non CMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>8_YT-_engagements</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:44:08</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/8_YT-_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Weeks presence per account</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>combine CMS &amp; non CMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>9_YT-_engagements</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:44:09</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>combine CMS &amp; non CMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>10_YT-_engagements</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:44:09</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>testing merge row count</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>combine CMS &amp; non CMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>6_YT-_engagements</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:44:08</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/6_YT-_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>all weeks in dataset</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>testing automated extracts</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>9_TWI_country</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:44:50</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/9_TWI_country_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>testing inner join - dataloss between two tables</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>checking country in lookup</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>10_TWI_country</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:44:50</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>testing missing elements in columns</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>stale country dataset - channels</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>9_YT-_country</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:52:54</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/9_YT-_country_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>testing missing elements in columns</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Check that all page IDs are found in SQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>10_YT-_country</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:52:54</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/10_YT-_country_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Weeks presence per account</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Check all weeks present for each account</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>11_YT-_country</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:52:55</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/11_YT-_country_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Check for NaN and positive values</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Check no missing values in page fans column from redshift returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>12_YT-_country</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:52:55</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Check no duplicates from redshift returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>13_YT-_country</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:52:55</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>testing inner join - dataloss between two tables</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>adding country codes GAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>14_YT-_country</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:52:55</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>testing inner join - dataloss between two tables</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>combining country and global views</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>15_YT-_country</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:52:55</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>testing country percentage</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>calculating % country</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>9_TWI_combination</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:57:10</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>10_TWI_combination</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:57:12</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/10_TWI_combination_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>testing inner join - dataloss between two tables</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>joining activity &amp; country - first</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>11_TWI_combination</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2025-11-23 10:57:12</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/11_TWI_combination_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>testing inner join - dataloss between two tables</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>joining activity &amp; country - second</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>9</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2025-11-23 11:07:26</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Testing if lookup DataFrame is empty</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring service is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>10</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2025-11-23 11:07:26</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring service is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>11</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2025-11-23 11:07:26</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Testing missing values in lookup</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>lookup files - ensuring service is correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1_YT_18</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2025-11-23 11:09:42</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/1_YT_18_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>testing inner join - dataloss between two tables</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>merging uv &amp; country</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>9_YT-_combination</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>2025-11-23 11:11:07</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/9_YT-_combination_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>testing inner join - dataloss between two tables</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>merging uv &amp; country</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>8_INS_engagements</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:40</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Check for NaN and positive values</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Check no missing values in metric columns from redshift returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>9_INS_engagements</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:40</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>no file created :)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>testing the combination of columns for uniqueness</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Check no duplicates from redshift returned</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>10_INS_engagements</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:40</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/10_INS_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>General outlier detection</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Check for extreme outliers in metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>11_INS_engagements</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2025-11-23 12:27:41</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>../test/issue_lists_2025-11-23/11_INS_engagements_issue_list.csv</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Upper-bound outlier detection vs reference</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Compare metrics to reference period</t>
         </is>
       </c>
     </row>

</xml_diff>